<commit_message>
Mise en forme finale des livrables du Projet I (cours d'Assurance Vie)
- Note technique : cadre « Assurance Vie », auteurs Groupe 1, superviseure
  Mme Fatou Diop ; suppression des tirets longs, de la section limites et
  de toute mention de simulation ; noms de fichiers retirés du texte ;
  cellules de tableaux sur une seule ligne ; lignes alternées orange/blanc
- Questionnaire : thème orange, en-tête au nom du groupe, consignes en
  lignes de tableau, grille sans retours à la ligne dans les cellules
- Simulateur : intitulés sans tirets longs, métadonnées d'auteur du groupe
- README actualisé

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01L8Gx8Yawmd4RBuYpXHqCkx
</commit_message>
<xml_diff>
--- a/Projet_IFC/simulateur_IFC_SENIA.xlsx
+++ b/Projet_IFC/simulateur_IFC_SENIA.xlsx
@@ -1,18 +1,18 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Hypotheses" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="BD" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Baremes" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Table_CIMA_H" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Calculs" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Resultats" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Hypotheses" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BD" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Baremes" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Table_CIMA_H" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Calculs" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resultats" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
     <definedName name="DateEval">Hypotheses!$B$6</definedName>
@@ -514,7 +514,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>SIMULATEUR IFC / IFC+ — ÉVALUATION ACTUARIELLE DU PASSIF SOCIAL</t>
+          <t>SIMULATEUR IFC / IFC+ : ÉVALUATION ACTUARIELLE DU PASSIF SOCIAL</t>
         </is>
       </c>
     </row>
@@ -526,7 +526,7 @@
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>SENIA S.A. — Sénégalaise des Industries Alimentaires</t>
+          <t>SENIA S.A. (Sénégalaise des Industries Alimentaires)</t>
         </is>
       </c>
     </row>
@@ -12059,7 +12059,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>SYNTHÈSE DE L'ÉVALUATION AU 31/12/2025 — SENIA S.A.</t>
+          <t>SYNTHÈSE DE L'ÉVALUATION AU 31/12/2025 : SENIA S.A.</t>
         </is>
       </c>
     </row>
@@ -12192,7 +12192,7 @@
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>Option 1 — Prime unique (engagement global + passif IL)</t>
+          <t>Option 1 : prime unique (engagement global + passif IL)</t>
         </is>
       </c>
       <c r="B17" s="21">
@@ -12203,7 +12203,7 @@
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>Option 2 — Prime initiale (dette actuarielle), puis charge normale annuelle</t>
+          <t>Option 2 : prime initiale (dette actuarielle), puis charge normale annuelle</t>
         </is>
       </c>
       <c r="B18" s="21">
@@ -12225,7 +12225,7 @@
     <row r="20">
       <c r="A20" s="9" t="inlineStr">
         <is>
-          <t>Option 3 — Amortissement de la dette actuarielle (par an)</t>
+          <t>Option 3 : amortissement de la dette actuarielle (par an)</t>
         </is>
       </c>
       <c r="B20" s="11">
@@ -12236,7 +12236,7 @@
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>Option 3 — Prime annuelle sur la durée d'amortissement</t>
+          <t>Option 3 : prime annuelle sur la durée d'amortissement</t>
         </is>
       </c>
       <c r="B21" s="21">

</xml_diff>